<commit_message>
Code after dry run completed for CZ new hires
</commit_message>
<xml_diff>
--- a/Data/testDataCzechia_PK17.xlsx
+++ b/Data/testDataCzechia_PK17.xlsx
@@ -3,13 +3,16 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27328"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{94ED81B8-6D36-446D-9F09-1C15C4E0BAAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:20001_{425DAAD6-BFB7-47E7-B5D1-90D9D47CCFA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1068" yWindow="-108" windowWidth="22080" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase">Sheet1!$A$1:$CA$16</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <fileRecoveryPr repairLoad="1"/>
   <extLst>
@@ -29,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="977" uniqueCount="224">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1016" uniqueCount="260">
   <si>
     <t>TestCaseIDs</t>
   </si>
@@ -256,7 +259,7 @@
     <t>ProposedPayGroupFinal</t>
   </si>
   <si>
-    <t>10697365</t>
+    <t>10697392</t>
   </si>
   <si>
     <t>Passed</t>
@@ -268,10 +271,10 @@
     <t>Czechia</t>
   </si>
   <si>
-    <t>Nikko</t>
-  </si>
-  <si>
-    <t>Abbott</t>
+    <t>Vella</t>
+  </si>
+  <si>
+    <t>Haag-Corwin</t>
   </si>
   <si>
     <t>770 272 784</t>
@@ -409,16 +412,19 @@
     <t>CZ Monthly</t>
   </si>
   <si>
+    <t>10697394</t>
+  </si>
+  <si>
     <t>895 Store Management (Sepap Pusube (10573442))</t>
   </si>
   <si>
-    <t>CzechiaTwo</t>
-  </si>
-  <si>
-    <t>PayrollTwentyFiveFebTwentySixD</t>
-  </si>
-  <si>
-    <t>Auto 56538241</t>
+    <t>Maximillia</t>
+  </si>
+  <si>
+    <t>Hills</t>
+  </si>
+  <si>
+    <t>Auto 36654543</t>
   </si>
   <si>
     <t>Department Manager_NEW</t>
@@ -436,7 +442,13 @@
     <t>Aina</t>
   </si>
   <si>
-    <t>CzechiaThree</t>
+    <t>10697395</t>
+  </si>
+  <si>
+    <t>Winona</t>
+  </si>
+  <si>
+    <t>Romaguera</t>
   </si>
   <si>
     <t>Fixed Term (Fixed Term)</t>
@@ -466,10 +478,16 @@
     <t>Ogbonda</t>
   </si>
   <si>
-    <t>CzechiaFour</t>
-  </si>
-  <si>
-    <t>Auto 50243455</t>
+    <t>10697410</t>
+  </si>
+  <si>
+    <t>Daphnee</t>
+  </si>
+  <si>
+    <t>Krajcik</t>
+  </si>
+  <si>
+    <t>Auto 88981386</t>
   </si>
   <si>
     <t>Assistant Store Manager_NEW</t>
@@ -490,16 +508,16 @@
     <t>Obot</t>
   </si>
   <si>
-    <t>Test failed for 'Maegan Jakubowski' Employee: Errors and AlertsErrorPage Error- You have not entered an amount within the Compensation Guidelines.     (Employee Compensation Event For Hire Employee)AlertPage Alert- "Warning: You have entered an amount that is outside of the range or more than 10% higher than the current salary.  Please re-enter an amount inside the range, below 10% or continue and it will be sent for approval."     (Employee Compensation Event For Hire Employee) &amp; find failed Screenshot Path:-&gt;H:\Latest_Workday_Playwright/WorkdayFailedScreenshot/2025-02-26T12-49-16-544Z.png</t>
+    <t>Test failed for 'Gregg Kunze' Employee: Errors and AlertsErrorPage Error- You have not entered an amount within the Compensation Guidelines.     (Employee Compensation Event For Hire Employee)AlertPage Alert- "Warning: You have entered an amount that is outside of the range or more than 10% higher than the current salary.  Please re-enter an amount inside the range, below 10% or continue and it will be sent for approval."     (Employee Compensation Event For Hire Employee) &amp; find failed Screenshot Path:-&gt;H:\Latest_Workday_Playwright/WorkdayFailedScreenshot/2025-02-27T05-27-26-153Z.png</t>
   </si>
   <si>
     <t>Failed</t>
   </si>
   <si>
-    <t>Maegan</t>
-  </si>
-  <si>
-    <t>Jakubowski</t>
+    <t>Gregg</t>
+  </si>
+  <si>
+    <t>Kunze</t>
   </si>
   <si>
     <t>Students</t>
@@ -526,13 +544,19 @@
     <t>Yusuf</t>
   </si>
   <si>
-    <t>CzechiaSix</t>
+    <t>10697396</t>
+  </si>
+  <si>
+    <t>Alicia</t>
+  </si>
+  <si>
+    <t>Heaney</t>
   </si>
   <si>
     <t>771 272 784</t>
   </si>
   <si>
-    <t>Auto 65008963</t>
+    <t>Auto 25082496</t>
   </si>
   <si>
     <t>In-Store Visual Merchandising Manager_NEW</t>
@@ -553,13 +577,13 @@
     <t>Torunarigha</t>
   </si>
   <si>
-    <t>10697367</t>
-  </si>
-  <si>
-    <t>Zachery</t>
-  </si>
-  <si>
-    <t>Hegmann</t>
+    <t>10697397</t>
+  </si>
+  <si>
+    <t>Garry</t>
+  </si>
+  <si>
+    <t>Jacobs</t>
   </si>
   <si>
     <t>772 272 784</t>
@@ -577,13 +601,19 @@
     <t>Ekong</t>
   </si>
   <si>
-    <t>CzechiaEight</t>
+    <t>10697398</t>
+  </si>
+  <si>
+    <t>Karolann</t>
+  </si>
+  <si>
+    <t>Wisozk</t>
   </si>
   <si>
     <t>773 272 784</t>
   </si>
   <si>
-    <t>Auto 74753275</t>
+    <t>Auto 38963605</t>
   </si>
   <si>
     <t>Store Manager_NEW</t>
@@ -595,7 +625,13 @@
     <t>Sanusi</t>
   </si>
   <si>
-    <t>CzechiaNine</t>
+    <t>10697411</t>
+  </si>
+  <si>
+    <t>Rupert</t>
+  </si>
+  <si>
+    <t>Schimmel</t>
   </si>
   <si>
     <t>774 272 784</t>
@@ -610,13 +646,16 @@
     <t>Ajayi</t>
   </si>
   <si>
-    <t>CzechiaTen</t>
+    <t>10697401</t>
+  </si>
+  <si>
+    <t>Barrows</t>
   </si>
   <si>
     <t>775 272 784</t>
   </si>
   <si>
-    <t>Auto 48421507</t>
+    <t>Auto 44247310</t>
   </si>
   <si>
     <t>Team Manager - Retail_NEW</t>
@@ -628,7 +667,13 @@
     <t>Awaziem</t>
   </si>
   <si>
-    <t>CzechiaEleven</t>
+    <t>10697402</t>
+  </si>
+  <si>
+    <t>Vaughn</t>
+  </si>
+  <si>
+    <t>Ebert</t>
   </si>
   <si>
     <t>776 272 784</t>
@@ -646,13 +691,19 @@
     <t>Ughelumba</t>
   </si>
   <si>
-    <t>CzechiaTwelve</t>
+    <t>10697404</t>
+  </si>
+  <si>
+    <t>Elinore</t>
+  </si>
+  <si>
+    <t>Aufderhar</t>
   </si>
   <si>
     <t>777 272 784</t>
   </si>
   <si>
-    <t>Auto 56536047</t>
+    <t>Auto 69175788</t>
   </si>
   <si>
     <t>In-Store P&amp;C Manager_NEW</t>
@@ -664,7 +715,13 @@
     <t>Ebuehi</t>
   </si>
   <si>
-    <t>CzechiaThirteen</t>
+    <t>10697405</t>
+  </si>
+  <si>
+    <t>Novella</t>
+  </si>
+  <si>
+    <t>Moore</t>
   </si>
   <si>
     <t>778 272 784</t>
@@ -679,7 +736,10 @@
     <t>Omeruo</t>
   </si>
   <si>
-    <t>CzechiaFourteen</t>
+    <t>10697412</t>
+  </si>
+  <si>
+    <t>Cyrus</t>
   </si>
   <si>
     <t>779 272 784</t>
@@ -691,7 +751,13 @@
     <t>Dele Bashiru</t>
   </si>
   <si>
-    <t>CzechiaFifteen</t>
+    <t>10697409</t>
+  </si>
+  <si>
+    <t>Kevin</t>
+  </si>
+  <si>
+    <t>Kiehn</t>
   </si>
   <si>
     <t>255 Stockroom</t>
@@ -701,6 +767,51 @@
   </si>
   <si>
     <t>Onovo</t>
+  </si>
+  <si>
+    <t>Test1</t>
+  </si>
+  <si>
+    <t>Test2</t>
+  </si>
+  <si>
+    <t>Test9</t>
+  </si>
+  <si>
+    <t>Test5</t>
+  </si>
+  <si>
+    <t>Test7</t>
+  </si>
+  <si>
+    <t>Test8</t>
+  </si>
+  <si>
+    <t>Test3</t>
+  </si>
+  <si>
+    <t>Test4</t>
+  </si>
+  <si>
+    <t>Test6</t>
+  </si>
+  <si>
+    <t>Test10</t>
+  </si>
+  <si>
+    <t>Test11</t>
+  </si>
+  <si>
+    <t>Test12</t>
+  </si>
+  <si>
+    <t>Test13</t>
+  </si>
+  <si>
+    <t>Test14</t>
+  </si>
+  <si>
+    <t>Test15</t>
   </si>
 </sst>
 </file>
@@ -710,7 +821,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="mm/dd/yyyy"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -755,6 +866,12 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -777,12 +894,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF00FF00"/>
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
+        <fgColor rgb="FF00FF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -826,7 +944,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -842,37 +960,40 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="14" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="4" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1496,7 +1617,9 @@
       <c r="CN1" s="1"/>
     </row>
     <row r="2" spans="1:92" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="8"/>
+      <c r="A2" s="8" t="s">
+        <v>245</v>
+      </c>
       <c r="B2" s="9" t="s">
         <v>75</v>
       </c>
@@ -1635,7 +1758,7 @@
         <v>103</v>
       </c>
       <c r="AT2" s="18">
-        <v>9661117554</v>
+        <v>9661111262</v>
       </c>
       <c r="AU2" s="13" t="s">
         <v>104</v>
@@ -1649,8 +1772,8 @@
       <c r="AX2" s="17" t="s">
         <v>106</v>
       </c>
-      <c r="AY2" s="18">
-        <v>144512746</v>
+      <c r="AY2" s="19">
+        <v>144062791</v>
       </c>
       <c r="AZ2" s="13" t="s">
         <v>104</v>
@@ -1738,20 +1861,26 @@
       </c>
     </row>
     <row r="3" spans="1:92" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="8"/>
-      <c r="B3" s="8"/>
-      <c r="C3" s="8"/>
+      <c r="A3" s="8" t="s">
+        <v>246</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>76</v>
+      </c>
       <c r="D3" s="10" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E3" s="11" t="s">
         <v>78</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="G3" s="12" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="H3" s="12" t="s">
         <v>81</v>
@@ -1809,13 +1938,13 @@
         <v>90</v>
       </c>
       <c r="Z3" s="12" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="AA3" s="8" t="s">
         <v>92</v>
       </c>
       <c r="AB3" s="8" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="AC3" s="8" t="s">
         <v>94</v>
@@ -1854,10 +1983,10 @@
         <v>45597</v>
       </c>
       <c r="AN3" s="12" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="AO3" s="8" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="AP3" s="11">
         <v>100</v>
@@ -1873,7 +2002,7 @@
         <v>103</v>
       </c>
       <c r="AT3" s="18">
-        <v>9661119083</v>
+        <v>9661119688</v>
       </c>
       <c r="AU3" s="13" t="s">
         <v>104</v>
@@ -1887,8 +2016,8 @@
       <c r="AX3" s="17" t="s">
         <v>106</v>
       </c>
-      <c r="AY3" s="18">
-        <v>144502747</v>
+      <c r="AY3" s="19">
+        <v>144052792</v>
       </c>
       <c r="AZ3" s="13" t="s">
         <v>104</v>
@@ -1957,10 +2086,10 @@
         <v>78</v>
       </c>
       <c r="BV3" s="14" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="BW3" s="14" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="BX3" s="14">
         <v>201</v>
@@ -1976,9 +2105,15 @@
       </c>
     </row>
     <row r="4" spans="1:92" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="8"/>
-      <c r="B4" s="8"/>
-      <c r="C4" s="8"/>
+      <c r="A4" s="8" t="s">
+        <v>251</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>136</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>76</v>
+      </c>
       <c r="D4" s="10" t="s">
         <v>77</v>
       </c>
@@ -1986,10 +2121,10 @@
         <v>78</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G4" s="12" t="s">
-        <v>128</v>
+        <v>138</v>
       </c>
       <c r="H4" s="12" t="s">
         <v>81</v>
@@ -2050,13 +2185,13 @@
         <v>91</v>
       </c>
       <c r="AA4" s="8" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="AB4" s="8" t="s">
         <v>93</v>
       </c>
       <c r="AC4" s="8" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="AD4" s="11" t="s">
         <v>95</v>
@@ -2065,7 +2200,7 @@
         <v>96</v>
       </c>
       <c r="AF4" s="8" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="AG4" s="16">
         <v>20</v>
@@ -2096,7 +2231,7 @@
         <v>101</v>
       </c>
       <c r="AO4" s="8" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="AP4" s="11">
         <v>100</v>
@@ -2112,7 +2247,7 @@
         <v>103</v>
       </c>
       <c r="AT4" s="18">
-        <v>9661111889</v>
+        <v>9661111955</v>
       </c>
       <c r="AU4" s="13" t="s">
         <v>104</v>
@@ -2126,8 +2261,8 @@
       <c r="AX4" s="17" t="s">
         <v>106</v>
       </c>
-      <c r="AY4" s="18">
-        <v>144492748</v>
+      <c r="AY4" s="19">
+        <v>144082789</v>
       </c>
       <c r="AZ4" s="13" t="s">
         <v>104</v>
@@ -2166,10 +2301,10 @@
         <v>78</v>
       </c>
       <c r="BL4" s="14" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="BM4" s="14" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="BN4" s="14" t="s">
         <v>117</v>
@@ -2187,7 +2322,7 @@
         <v>1991</v>
       </c>
       <c r="BS4" s="14" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="BT4" s="14" t="s">
         <v>120</v>
@@ -2196,10 +2331,10 @@
         <v>78</v>
       </c>
       <c r="BV4" s="14" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="BW4" s="14" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="BX4" s="14">
         <v>213</v>
@@ -2215,20 +2350,26 @@
       </c>
     </row>
     <row r="5" spans="1:92" s="7" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="8"/>
-      <c r="B5" s="8"/>
-      <c r="C5" s="8"/>
+      <c r="A5" s="8" t="s">
+        <v>252</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>148</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>76</v>
+      </c>
       <c r="D5" s="10" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E5" s="11" t="s">
         <v>78</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="G5" s="12" t="s">
-        <v>128</v>
+        <v>150</v>
       </c>
       <c r="H5" s="12" t="s">
         <v>81</v>
@@ -2286,13 +2427,13 @@
         <v>90</v>
       </c>
       <c r="Z5" s="12" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="AA5" s="8" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="AB5" s="8" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="AC5" s="8" t="s">
         <v>94</v>
@@ -2332,10 +2473,10 @@
         <v>45597</v>
       </c>
       <c r="AN5" s="12" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="AO5" s="8" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="AP5" s="11">
         <v>100</v>
@@ -2351,7 +2492,7 @@
         <v>103</v>
       </c>
       <c r="AT5" s="18">
-        <v>9661115607</v>
+        <v>9661117752</v>
       </c>
       <c r="AU5" s="13" t="s">
         <v>104</v>
@@ -2365,8 +2506,8 @@
       <c r="AX5" s="17" t="s">
         <v>106</v>
       </c>
-      <c r="AY5" s="18">
-        <v>144482749</v>
+      <c r="AY5" s="19">
+        <v>144072790</v>
       </c>
       <c r="AZ5" s="13" t="s">
         <v>104</v>
@@ -2405,10 +2546,10 @@
         <v>78</v>
       </c>
       <c r="BL5" s="14" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="BM5" s="14" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="BN5" s="14" t="s">
         <v>117</v>
@@ -2426,7 +2567,7 @@
         <v>2024</v>
       </c>
       <c r="BS5" s="14" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="BT5" s="14" t="s">
         <v>120</v>
@@ -2435,10 +2576,10 @@
         <v>78</v>
       </c>
       <c r="BV5" s="14" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="BW5" s="14" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="BX5" s="14">
         <v>207</v>
@@ -2454,12 +2595,14 @@
       </c>
     </row>
     <row r="6" spans="1:92" s="7" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="8"/>
+      <c r="A6" s="8" t="s">
+        <v>248</v>
+      </c>
       <c r="B6" s="8" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="D6" s="10" t="s">
         <v>77</v>
@@ -2468,10 +2611,10 @@
         <v>78</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="G6" s="12" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="H6" s="12" t="s">
         <v>81</v>
@@ -2532,22 +2675,22 @@
         <v>91</v>
       </c>
       <c r="AA6" s="8" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="AB6" s="8" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="AC6" s="8" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="AD6" s="11" t="s">
         <v>95</v>
       </c>
       <c r="AE6" s="11" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="AF6" s="8" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="AG6" s="16">
         <v>16</v>
@@ -2557,7 +2700,7 @@
         <v>45962</v>
       </c>
       <c r="AI6" s="12" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="AJ6" s="12" t="s">
         <v>100</v>
@@ -2578,7 +2721,7 @@
         <v>101</v>
       </c>
       <c r="AO6" s="8" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="AP6" s="11">
         <v>100</v>
@@ -2594,7 +2737,7 @@
         <v>103</v>
       </c>
       <c r="AT6" s="18">
-        <v>9661118423</v>
+        <v>9661110921</v>
       </c>
       <c r="AU6" s="13" t="s">
         <v>104</v>
@@ -2609,7 +2752,7 @@
         <v>106</v>
       </c>
       <c r="AY6" s="18">
-        <v>144472750</v>
+        <v>144322765</v>
       </c>
       <c r="AZ6" s="13" t="s">
         <v>104</v>
@@ -2678,10 +2821,10 @@
         <v>78</v>
       </c>
       <c r="BV6" s="14" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="BW6" s="14" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="BX6" s="14">
         <v>211</v>
@@ -2697,23 +2840,29 @@
       </c>
     </row>
     <row r="7" spans="1:92" s="7" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="8"/>
-      <c r="B7" s="8"/>
-      <c r="C7" s="8"/>
+      <c r="A7" s="8" t="s">
+        <v>253</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>170</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>76</v>
+      </c>
       <c r="D7" s="10" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E7" s="11" t="s">
         <v>78</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>165</v>
+        <v>171</v>
       </c>
       <c r="G7" s="12" t="s">
-        <v>128</v>
+        <v>172</v>
       </c>
       <c r="H7" s="12" t="s">
-        <v>166</v>
+        <v>173</v>
       </c>
       <c r="I7" s="12" t="s">
         <v>82</v>
@@ -2768,16 +2917,16 @@
         <v>90</v>
       </c>
       <c r="Z7" s="12" t="s">
-        <v>167</v>
+        <v>174</v>
       </c>
       <c r="AA7" s="8" t="s">
         <v>92</v>
       </c>
       <c r="AB7" s="8" t="s">
-        <v>168</v>
+        <v>175</v>
       </c>
       <c r="AC7" s="8" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="AD7" s="11" t="s">
         <v>95</v>
@@ -2813,10 +2962,10 @@
         <v>45597</v>
       </c>
       <c r="AN7" s="12" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="AO7" s="8" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="AP7" s="11">
         <v>100</v>
@@ -2832,7 +2981,7 @@
         <v>103</v>
       </c>
       <c r="AT7" s="18">
-        <v>9661118412</v>
+        <v>9661116410</v>
       </c>
       <c r="AU7" s="13" t="s">
         <v>104</v>
@@ -2847,7 +2996,7 @@
         <v>106</v>
       </c>
       <c r="AY7" s="18">
-        <v>144462751</v>
+        <v>144202777</v>
       </c>
       <c r="AZ7" s="13" t="s">
         <v>104</v>
@@ -2886,10 +3035,10 @@
         <v>78</v>
       </c>
       <c r="BL7" s="14" t="s">
-        <v>169</v>
+        <v>176</v>
       </c>
       <c r="BM7" s="14" t="s">
-        <v>170</v>
+        <v>177</v>
       </c>
       <c r="BN7" s="14" t="s">
         <v>117</v>
@@ -2907,7 +3056,7 @@
         <v>2000</v>
       </c>
       <c r="BS7" s="14" t="s">
-        <v>171</v>
+        <v>178</v>
       </c>
       <c r="BT7" s="14" t="s">
         <v>120</v>
@@ -2916,10 +3065,10 @@
         <v>78</v>
       </c>
       <c r="BV7" s="14" t="s">
-        <v>172</v>
+        <v>179</v>
       </c>
       <c r="BW7" s="14" t="s">
-        <v>173</v>
+        <v>180</v>
       </c>
       <c r="BX7" s="14">
         <v>211</v>
@@ -2935,9 +3084,11 @@
       </c>
     </row>
     <row r="8" spans="1:92" s="7" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="8"/>
+      <c r="A8" s="8" t="s">
+        <v>249</v>
+      </c>
       <c r="B8" s="8" t="s">
-        <v>174</v>
+        <v>181</v>
       </c>
       <c r="C8" s="8" t="s">
         <v>76</v>
@@ -2949,13 +3100,13 @@
         <v>78</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>175</v>
+        <v>182</v>
       </c>
       <c r="G8" s="12" t="s">
-        <v>176</v>
+        <v>183</v>
       </c>
       <c r="H8" s="12" t="s">
-        <v>177</v>
+        <v>184</v>
       </c>
       <c r="I8" s="12" t="s">
         <v>82</v>
@@ -3013,13 +3164,13 @@
         <v>91</v>
       </c>
       <c r="AA8" s="8" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="AB8" s="8" t="s">
-        <v>178</v>
+        <v>185</v>
       </c>
       <c r="AC8" s="8" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="AD8" s="11" t="s">
         <v>95</v>
@@ -3059,7 +3210,7 @@
         <v>101</v>
       </c>
       <c r="AO8" s="8" t="s">
-        <v>179</v>
+        <v>186</v>
       </c>
       <c r="AP8" s="11">
         <v>100</v>
@@ -3075,7 +3226,7 @@
         <v>103</v>
       </c>
       <c r="AT8" s="18">
-        <v>9661118973</v>
+        <v>9661117444</v>
       </c>
       <c r="AU8" s="13" t="s">
         <v>104</v>
@@ -3090,7 +3241,7 @@
         <v>106</v>
       </c>
       <c r="AY8" s="18">
-        <v>144452752</v>
+        <v>144302767</v>
       </c>
       <c r="AZ8" s="13" t="s">
         <v>104</v>
@@ -3159,10 +3310,10 @@
         <v>78</v>
       </c>
       <c r="BV8" s="14" t="s">
-        <v>180</v>
+        <v>187</v>
       </c>
       <c r="BW8" s="14" t="s">
-        <v>181</v>
+        <v>188</v>
       </c>
       <c r="BX8" s="14">
         <v>213</v>
@@ -3178,23 +3329,29 @@
       </c>
     </row>
     <row r="9" spans="1:92" s="7" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="8"/>
-      <c r="B9" s="8"/>
-      <c r="C9" s="8"/>
+      <c r="A9" s="8" t="s">
+        <v>250</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>189</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>76</v>
+      </c>
       <c r="D9" s="10" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E9" s="11" t="s">
         <v>78</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>182</v>
+        <v>190</v>
       </c>
       <c r="G9" s="12" t="s">
-        <v>128</v>
+        <v>191</v>
       </c>
       <c r="H9" s="12" t="s">
-        <v>183</v>
+        <v>192</v>
       </c>
       <c r="I9" s="12" t="s">
         <v>82</v>
@@ -3249,13 +3406,13 @@
         <v>90</v>
       </c>
       <c r="Z9" s="12" t="s">
-        <v>184</v>
+        <v>193</v>
       </c>
       <c r="AA9" s="8" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="AB9" s="8" t="s">
-        <v>185</v>
+        <v>194</v>
       </c>
       <c r="AC9" s="8" t="s">
         <v>94</v>
@@ -3295,10 +3452,10 @@
         <v>45597</v>
       </c>
       <c r="AN9" s="12" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="AO9" s="8" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="AP9" s="11">
         <v>100</v>
@@ -3314,7 +3471,7 @@
         <v>103</v>
       </c>
       <c r="AT9" s="18">
-        <v>9661114815</v>
+        <v>9661119908</v>
       </c>
       <c r="AU9" s="13" t="s">
         <v>104</v>
@@ -3329,7 +3486,7 @@
         <v>106</v>
       </c>
       <c r="AY9" s="18">
-        <v>144442753</v>
+        <v>144192778</v>
       </c>
       <c r="AZ9" s="13" t="s">
         <v>104</v>
@@ -3368,10 +3525,10 @@
         <v>78</v>
       </c>
       <c r="BL9" s="14" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="BM9" s="14" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="BN9" s="14" t="s">
         <v>117</v>
@@ -3389,7 +3546,7 @@
         <v>1991</v>
       </c>
       <c r="BS9" s="14" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="BT9" s="14" t="s">
         <v>120</v>
@@ -3398,10 +3555,10 @@
         <v>78</v>
       </c>
       <c r="BV9" s="14" t="s">
-        <v>186</v>
+        <v>195</v>
       </c>
       <c r="BW9" s="14" t="s">
-        <v>187</v>
+        <v>196</v>
       </c>
       <c r="BX9" s="14">
         <v>211</v>
@@ -3417,9 +3574,15 @@
       </c>
     </row>
     <row r="10" spans="1:92" s="7" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="8"/>
-      <c r="B10" s="8"/>
-      <c r="C10" s="8"/>
+      <c r="A10" s="8" t="s">
+        <v>247</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>197</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>76</v>
+      </c>
       <c r="D10" s="10" t="s">
         <v>77</v>
       </c>
@@ -3427,13 +3590,13 @@
         <v>78</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>188</v>
+        <v>198</v>
       </c>
       <c r="G10" s="12" t="s">
-        <v>128</v>
+        <v>199</v>
       </c>
       <c r="H10" s="12" t="s">
-        <v>189</v>
+        <v>200</v>
       </c>
       <c r="I10" s="12" t="s">
         <v>82</v>
@@ -3494,10 +3657,10 @@
         <v>92</v>
       </c>
       <c r="AB10" s="8" t="s">
-        <v>190</v>
+        <v>201</v>
       </c>
       <c r="AC10" s="8" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="AD10" s="11" t="s">
         <v>95</v>
@@ -3506,7 +3669,7 @@
         <v>96</v>
       </c>
       <c r="AF10" s="8" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="AG10" s="16">
         <v>20</v>
@@ -3536,7 +3699,7 @@
         <v>101</v>
       </c>
       <c r="AO10" s="8" t="s">
-        <v>179</v>
+        <v>186</v>
       </c>
       <c r="AP10" s="11">
         <v>100</v>
@@ -3552,7 +3715,7 @@
         <v>103</v>
       </c>
       <c r="AT10" s="18">
-        <v>9661115728</v>
+        <v>9661111757</v>
       </c>
       <c r="AU10" s="13" t="s">
         <v>104</v>
@@ -3567,7 +3730,7 @@
         <v>106</v>
       </c>
       <c r="AY10" s="18">
-        <v>144432754</v>
+        <v>144282769</v>
       </c>
       <c r="AZ10" s="13" t="s">
         <v>104</v>
@@ -3606,10 +3769,10 @@
         <v>78</v>
       </c>
       <c r="BL10" s="14" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="BM10" s="14" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="BN10" s="14" t="s">
         <v>117</v>
@@ -3627,7 +3790,7 @@
         <v>2024</v>
       </c>
       <c r="BS10" s="14" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="BT10" s="14" t="s">
         <v>120</v>
@@ -3636,10 +3799,10 @@
         <v>78</v>
       </c>
       <c r="BV10" s="14" t="s">
-        <v>191</v>
+        <v>202</v>
       </c>
       <c r="BW10" s="14" t="s">
-        <v>192</v>
+        <v>203</v>
       </c>
       <c r="BX10" s="14">
         <v>213</v>
@@ -3655,23 +3818,29 @@
       </c>
     </row>
     <row r="11" spans="1:92" s="7" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="8"/>
-      <c r="B11" s="8"/>
-      <c r="C11" s="8"/>
+      <c r="A11" s="8" t="s">
+        <v>254</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>204</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>76</v>
+      </c>
       <c r="D11" s="10" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E11" s="11" t="s">
         <v>78</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>193</v>
+        <v>182</v>
       </c>
       <c r="G11" s="12" t="s">
-        <v>128</v>
+        <v>205</v>
       </c>
       <c r="H11" s="12" t="s">
-        <v>194</v>
+        <v>206</v>
       </c>
       <c r="I11" s="12" t="s">
         <v>82</v>
@@ -3726,13 +3895,13 @@
         <v>90</v>
       </c>
       <c r="Z11" s="12" t="s">
-        <v>195</v>
+        <v>207</v>
       </c>
       <c r="AA11" s="8" t="s">
         <v>92</v>
       </c>
       <c r="AB11" s="8" t="s">
-        <v>196</v>
+        <v>208</v>
       </c>
       <c r="AC11" s="8" t="s">
         <v>94</v>
@@ -3771,10 +3940,10 @@
         <v>45597</v>
       </c>
       <c r="AN11" s="12" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="AO11" s="8" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="AP11" s="11">
         <v>100</v>
@@ -3790,7 +3959,7 @@
         <v>103</v>
       </c>
       <c r="AT11" s="18">
-        <v>9661119930</v>
+        <v>9661111933</v>
       </c>
       <c r="AU11" s="13" t="s">
         <v>104</v>
@@ -3805,7 +3974,7 @@
         <v>106</v>
       </c>
       <c r="AY11" s="18">
-        <v>144422755</v>
+        <v>144182779</v>
       </c>
       <c r="AZ11" s="13" t="s">
         <v>104</v>
@@ -3874,10 +4043,10 @@
         <v>78</v>
       </c>
       <c r="BV11" s="14" t="s">
-        <v>197</v>
+        <v>209</v>
       </c>
       <c r="BW11" s="14" t="s">
-        <v>198</v>
+        <v>210</v>
       </c>
       <c r="BX11" s="14">
         <v>201</v>
@@ -3893,9 +4062,15 @@
       </c>
     </row>
     <row r="12" spans="1:92" s="7" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="8"/>
-      <c r="B12" s="8"/>
-      <c r="C12" s="8"/>
+      <c r="A12" s="8" t="s">
+        <v>255</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>211</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>76</v>
+      </c>
       <c r="D12" s="10" t="s">
         <v>77</v>
       </c>
@@ -3903,13 +4078,13 @@
         <v>78</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>199</v>
+        <v>212</v>
       </c>
       <c r="G12" s="12" t="s">
-        <v>128</v>
+        <v>213</v>
       </c>
       <c r="H12" s="12" t="s">
-        <v>200</v>
+        <v>214</v>
       </c>
       <c r="I12" s="12" t="s">
         <v>82</v>
@@ -3967,13 +4142,13 @@
         <v>91</v>
       </c>
       <c r="AA12" s="8" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="AB12" s="8" t="s">
-        <v>201</v>
+        <v>215</v>
       </c>
       <c r="AC12" s="8" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="AD12" s="11" t="s">
         <v>95</v>
@@ -4013,7 +4188,7 @@
         <v>101</v>
       </c>
       <c r="AO12" s="8" t="s">
-        <v>202</v>
+        <v>216</v>
       </c>
       <c r="AP12" s="11">
         <v>100</v>
@@ -4029,7 +4204,7 @@
         <v>103</v>
       </c>
       <c r="AT12" s="18">
-        <v>9661117169</v>
+        <v>9661118533</v>
       </c>
       <c r="AU12" s="13" t="s">
         <v>104</v>
@@ -4044,7 +4219,7 @@
         <v>106</v>
       </c>
       <c r="AY12" s="18">
-        <v>144412756</v>
+        <v>144262771</v>
       </c>
       <c r="AZ12" s="13" t="s">
         <v>104</v>
@@ -4083,10 +4258,10 @@
         <v>78</v>
       </c>
       <c r="BL12" s="14" t="s">
-        <v>169</v>
+        <v>176</v>
       </c>
       <c r="BM12" s="14" t="s">
-        <v>170</v>
+        <v>177</v>
       </c>
       <c r="BN12" s="14" t="s">
         <v>117</v>
@@ -4104,7 +4279,7 @@
         <v>2000</v>
       </c>
       <c r="BS12" s="14" t="s">
-        <v>171</v>
+        <v>178</v>
       </c>
       <c r="BT12" s="14" t="s">
         <v>120</v>
@@ -4113,10 +4288,10 @@
         <v>78</v>
       </c>
       <c r="BV12" s="14" t="s">
-        <v>203</v>
+        <v>217</v>
       </c>
       <c r="BW12" s="14" t="s">
-        <v>204</v>
+        <v>218</v>
       </c>
       <c r="BX12" s="14">
         <v>213</v>
@@ -4132,23 +4307,29 @@
       </c>
     </row>
     <row r="13" spans="1:92" s="7" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="8"/>
-      <c r="B13" s="8"/>
-      <c r="C13" s="8"/>
+      <c r="A13" s="8" t="s">
+        <v>256</v>
+      </c>
+      <c r="B13" s="8" t="s">
+        <v>219</v>
+      </c>
+      <c r="C13" s="8" t="s">
+        <v>76</v>
+      </c>
       <c r="D13" s="10" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E13" s="11" t="s">
         <v>78</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>205</v>
+        <v>220</v>
       </c>
       <c r="G13" s="12" t="s">
-        <v>128</v>
+        <v>221</v>
       </c>
       <c r="H13" s="12" t="s">
-        <v>206</v>
+        <v>222</v>
       </c>
       <c r="I13" s="12" t="s">
         <v>82</v>
@@ -4203,13 +4384,13 @@
         <v>90</v>
       </c>
       <c r="Z13" s="12" t="s">
-        <v>207</v>
+        <v>223</v>
       </c>
       <c r="AA13" s="8" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="AB13" s="8" t="s">
-        <v>208</v>
+        <v>224</v>
       </c>
       <c r="AC13" s="8" t="s">
         <v>94</v>
@@ -4249,10 +4430,10 @@
         <v>45597</v>
       </c>
       <c r="AN13" s="12" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="AO13" s="8" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="AP13" s="11">
         <v>100</v>
@@ -4268,7 +4449,7 @@
         <v>103</v>
       </c>
       <c r="AT13" s="18">
-        <v>9661110316</v>
+        <v>9661112560</v>
       </c>
       <c r="AU13" s="13" t="s">
         <v>104</v>
@@ -4283,7 +4464,7 @@
         <v>106</v>
       </c>
       <c r="AY13" s="18">
-        <v>144402757</v>
+        <v>144252772</v>
       </c>
       <c r="AZ13" s="13" t="s">
         <v>104</v>
@@ -4352,10 +4533,10 @@
         <v>78</v>
       </c>
       <c r="BV13" s="14" t="s">
-        <v>209</v>
+        <v>225</v>
       </c>
       <c r="BW13" s="14" t="s">
-        <v>210</v>
+        <v>226</v>
       </c>
       <c r="BX13" s="14">
         <v>209</v>
@@ -4371,9 +4552,15 @@
       </c>
     </row>
     <row r="14" spans="1:92" s="7" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="8"/>
-      <c r="B14" s="8"/>
-      <c r="C14" s="8"/>
+      <c r="A14" s="8" t="s">
+        <v>257</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>227</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>76</v>
+      </c>
       <c r="D14" s="10" t="s">
         <v>77</v>
       </c>
@@ -4381,13 +4568,13 @@
         <v>78</v>
       </c>
       <c r="F14" s="8" t="s">
-        <v>211</v>
+        <v>228</v>
       </c>
       <c r="G14" s="12" t="s">
-        <v>128</v>
+        <v>229</v>
       </c>
       <c r="H14" s="12" t="s">
-        <v>212</v>
+        <v>230</v>
       </c>
       <c r="I14" s="12" t="s">
         <v>82</v>
@@ -4448,10 +4635,10 @@
         <v>92</v>
       </c>
       <c r="AB14" s="8" t="s">
-        <v>190</v>
+        <v>201</v>
       </c>
       <c r="AC14" s="8" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="AD14" s="11" t="s">
         <v>95</v>
@@ -4460,7 +4647,7 @@
         <v>96</v>
       </c>
       <c r="AF14" s="8" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="AG14" s="16">
         <v>24</v>
@@ -4490,7 +4677,7 @@
         <v>101</v>
       </c>
       <c r="AO14" s="8" t="s">
-        <v>213</v>
+        <v>231</v>
       </c>
       <c r="AP14" s="11">
         <v>100</v>
@@ -4506,7 +4693,7 @@
         <v>103</v>
       </c>
       <c r="AT14" s="18">
-        <v>9661115200</v>
+        <v>9661110338</v>
       </c>
       <c r="AU14" s="13" t="s">
         <v>104</v>
@@ -4521,7 +4708,7 @@
         <v>106</v>
       </c>
       <c r="AY14" s="18">
-        <v>144392758</v>
+        <v>144242773</v>
       </c>
       <c r="AZ14" s="13" t="s">
         <v>104</v>
@@ -4560,10 +4747,10 @@
         <v>78</v>
       </c>
       <c r="BL14" s="14" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="BM14" s="14" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="BN14" s="14" t="s">
         <v>117</v>
@@ -4581,7 +4768,7 @@
         <v>1991</v>
       </c>
       <c r="BS14" s="14" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="BT14" s="14" t="s">
         <v>120</v>
@@ -4590,10 +4777,10 @@
         <v>78</v>
       </c>
       <c r="BV14" s="14" t="s">
-        <v>214</v>
+        <v>232</v>
       </c>
       <c r="BW14" s="14" t="s">
-        <v>215</v>
+        <v>233</v>
       </c>
       <c r="BX14" s="14">
         <v>211</v>
@@ -4609,9 +4796,15 @@
       </c>
     </row>
     <row r="15" spans="1:92" s="7" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="8"/>
-      <c r="B15" s="8"/>
-      <c r="C15" s="8"/>
+      <c r="A15" s="8" t="s">
+        <v>258</v>
+      </c>
+      <c r="B15" s="8" t="s">
+        <v>234</v>
+      </c>
+      <c r="C15" s="8" t="s">
+        <v>76</v>
+      </c>
       <c r="D15" s="10" t="s">
         <v>77</v>
       </c>
@@ -4619,13 +4812,13 @@
         <v>78</v>
       </c>
       <c r="F15" s="8" t="s">
-        <v>216</v>
+        <v>235</v>
       </c>
       <c r="G15" s="12" t="s">
-        <v>128</v>
+        <v>191</v>
       </c>
       <c r="H15" s="12" t="s">
-        <v>217</v>
+        <v>236</v>
       </c>
       <c r="I15" s="12" t="s">
         <v>82</v>
@@ -4683,10 +4876,10 @@
         <v>91</v>
       </c>
       <c r="AA15" s="8" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="AB15" s="8" t="s">
-        <v>190</v>
+        <v>201</v>
       </c>
       <c r="AC15" s="8" t="s">
         <v>94</v>
@@ -4729,7 +4922,7 @@
         <v>101</v>
       </c>
       <c r="AO15" s="8" t="s">
-        <v>179</v>
+        <v>186</v>
       </c>
       <c r="AP15" s="11">
         <v>100</v>
@@ -4745,7 +4938,7 @@
         <v>103</v>
       </c>
       <c r="AT15" s="18">
-        <v>9661111647</v>
+        <v>9661118511</v>
       </c>
       <c r="AU15" s="13" t="s">
         <v>104</v>
@@ -4760,7 +4953,7 @@
         <v>106</v>
       </c>
       <c r="AY15" s="18">
-        <v>144382759</v>
+        <v>144232774</v>
       </c>
       <c r="AZ15" s="13" t="s">
         <v>104</v>
@@ -4799,10 +4992,10 @@
         <v>78</v>
       </c>
       <c r="BL15" s="14" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="BM15" s="14" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="BN15" s="14" t="s">
         <v>117</v>
@@ -4820,7 +5013,7 @@
         <v>2024</v>
       </c>
       <c r="BS15" s="14" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="BT15" s="14" t="s">
         <v>120</v>
@@ -4829,10 +5022,10 @@
         <v>78</v>
       </c>
       <c r="BV15" s="14" t="s">
-        <v>218</v>
+        <v>237</v>
       </c>
       <c r="BW15" s="14" t="s">
-        <v>219</v>
+        <v>238</v>
       </c>
       <c r="BX15" s="14">
         <v>213</v>
@@ -4848,9 +5041,15 @@
       </c>
     </row>
     <row r="16" spans="1:92" s="7" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="8"/>
-      <c r="B16" s="8"/>
-      <c r="C16" s="8"/>
+      <c r="A16" s="8" t="s">
+        <v>259</v>
+      </c>
+      <c r="B16" s="8" t="s">
+        <v>239</v>
+      </c>
+      <c r="C16" s="8" t="s">
+        <v>76</v>
+      </c>
       <c r="D16" s="10" t="s">
         <v>77</v>
       </c>
@@ -4858,13 +5057,13 @@
         <v>78</v>
       </c>
       <c r="F16" s="8" t="s">
-        <v>220</v>
+        <v>240</v>
       </c>
       <c r="G16" s="12" t="s">
-        <v>128</v>
+        <v>241</v>
       </c>
       <c r="H16" s="12" t="s">
-        <v>217</v>
+        <v>236</v>
       </c>
       <c r="I16" s="12" t="s">
         <v>82</v>
@@ -4928,7 +5127,7 @@
         <v>93</v>
       </c>
       <c r="AC16" s="8" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="AD16" s="11" t="s">
         <v>95</v>
@@ -4967,7 +5166,7 @@
         <v>101</v>
       </c>
       <c r="AO16" s="8" t="s">
-        <v>221</v>
+        <v>242</v>
       </c>
       <c r="AP16" s="11">
         <v>100</v>
@@ -4983,7 +5182,7 @@
         <v>103</v>
       </c>
       <c r="AT16" s="18">
-        <v>9661118610</v>
+        <v>9661117620</v>
       </c>
       <c r="AU16" s="13" t="s">
         <v>104</v>
@@ -4998,7 +5197,7 @@
         <v>106</v>
       </c>
       <c r="AY16" s="18">
-        <v>144372760</v>
+        <v>144222775</v>
       </c>
       <c r="AZ16" s="13" t="s">
         <v>104</v>
@@ -5037,10 +5236,10 @@
         <v>78</v>
       </c>
       <c r="BL16" s="14" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="BM16" s="14" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="BN16" s="14" t="s">
         <v>117</v>
@@ -5058,7 +5257,7 @@
         <v>2024</v>
       </c>
       <c r="BS16" s="14" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="BT16" s="14" t="s">
         <v>120</v>
@@ -5067,10 +5266,10 @@
         <v>78</v>
       </c>
       <c r="BV16" s="14" t="s">
-        <v>222</v>
+        <v>243</v>
       </c>
       <c r="BW16" s="14" t="s">
-        <v>223</v>
+        <v>244</v>
       </c>
       <c r="BX16" s="14">
         <v>211</v>
@@ -5086,6 +5285,7 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="7" type="noConversion"/>
   <dataValidations count="4">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AJ10:AJ16 Y10:Y16 W10:W16 T10:T16" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>INDIRECT($D1)</formula1>

</xml_diff>